<commit_message>
updated column headers of summary section
</commit_message>
<xml_diff>
--- a/rx_MiniMall_AutoPayReport.xlsx
+++ b/rx_MiniMall_AutoPayReport.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yardi365-my.sharepoint.com/personal/beril_pehlivan_yardi_com/Documents/Storage/Avenue-MiniMall/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yardi365-my.sharepoint.com/personal/beril_pehlivan_yardi_com/Documents/Storage/Avenue-MiniMall/MM-AutoPayYSR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{AD45799E-F075-40D4-9DE4-3EDACB2FABDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C794BC5-C3F9-47C0-9B6F-37E448A1437D}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="8_{AD45799E-F075-40D4-9DE4-3EDACB2FABDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CC6630E-0554-48CB-9C73-3DECCC22AAC1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{BCDFC48E-5E53-4A23-9E52-6F029E0D0EF1}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BCDFC48E-5E53-4A23-9E52-6F029E0D0EF1}"/>
   </bookViews>
   <sheets>
     <sheet name="rpt" sheetId="1" r:id="rId1"/>
@@ -41,15 +41,9 @@
     <t>Tenant Auto Pay Report</t>
   </si>
   <si>
-    <t>Name First/Last</t>
-  </si>
-  <si>
     <t>Unit #</t>
   </si>
   <si>
-    <t>EXP. Date</t>
-  </si>
-  <si>
     <t>Last 4 of Card</t>
   </si>
   <si>
@@ -62,9 +56,6 @@
     <t>Pending Charge Date</t>
   </si>
   <si>
-    <t>Total on Auto Pay</t>
-  </si>
-  <si>
     <t>Total Exp in 28 Days</t>
   </si>
   <si>
@@ -129,12 +120,25 @@
   </si>
   <si>
     <t>&amp;=APSum.PropName</t>
+  </si>
+  <si>
+    <t>Tenant Name</t>
+  </si>
+  <si>
+    <t>Auto Pay Stop Date</t>
+  </si>
+  <si>
+    <t>Total Tenants on Auto Pay</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -220,15 +224,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -567,131 +587,131 @@
   <dimension ref="A1:H10"/>
   <sheetFormatPr defaultColWidth="20.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.81640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="20.7265625" style="1"/>
+    <col min="1" max="1" width="20.7265625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="13.1796875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="17" style="3" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.81640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="19.90625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="20.7265625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="6" t="s">
         <v>5</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="E4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="F4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>19</v>
-      </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="2" t="s">
+    <row r="9" spans="1:8" s="8" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="A9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="H9" s="6" t="s">
         <v>9</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="A10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="1" t="s">
+      <c r="F10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="G10" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>27</v>
+      <c r="H10" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixes for Summary to Excel to show stacked on one page
</commit_message>
<xml_diff>
--- a/rx_MiniMall_AutoPayReport.xlsx
+++ b/rx_MiniMall_AutoPayReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://yardi365-my.sharepoint.com/personal/beril_pehlivan_yardi_com/Documents/Storage/Avenue-MiniMall/MM-AutoPayYSR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="8_{AD45799E-F075-40D4-9DE4-3EDACB2FABDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CC6630E-0554-48CB-9C73-3DECCC22AAC1}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="8_{AD45799E-F075-40D4-9DE4-3EDACB2FABDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1821414-B2AB-4E17-BA34-80909DF44686}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{BCDFC48E-5E53-4A23-9E52-6F029E0D0EF1}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{BCDFC48E-5E53-4A23-9E52-6F029E0D0EF1}"/>
   </bookViews>
   <sheets>
     <sheet name="rpt" sheetId="1" r:id="rId1"/>
@@ -62,9 +62,6 @@
     <t># of CC on Auto Pay</t>
   </si>
   <si>
-    <t>Total Billed</t>
-  </si>
-  <si>
     <t>Total Pending Charges</t>
   </si>
   <si>
@@ -129,6 +126,9 @@
   </si>
   <si>
     <t>Total Tenants on Auto Pay</t>
+  </si>
+  <si>
+    <t>Total Last Billed</t>
   </si>
 </sst>
 </file>
@@ -139,7 +139,7 @@
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,14 +161,20 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
-      <sz val="11"/>
+      <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -187,13 +193,43 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.249977111117893"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.249977111117893"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -206,49 +242,47 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -584,134 +618,137 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0BD3FF0-16FC-4ECE-ABDB-6EAEB8607F02}">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultColWidth="20.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.7265625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="13.1796875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="17" style="3" customWidth="1"/>
-    <col min="4" max="4" width="17.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.81640625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="19.90625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.81640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="20.7265625" style="3"/>
+    <col min="1" max="1" width="27.453125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="13.1796875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="17" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.81640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="20.7265625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:8" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+    </row>
+    <row r="3" spans="1:8" s="3" customFormat="1" ht="12" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="5"/>
+    </row>
+    <row r="5" spans="1:8" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:8" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:8" s="3" customFormat="1" ht="24" x14ac:dyDescent="0.35">
+      <c r="A7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="B7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="3" t="s">
+    <row r="8" spans="1:8" s="2" customFormat="1" ht="12" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" s="8" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F9" s="6" t="s">
+      <c r="C8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" s="3" t="s">
+      <c r="G8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="H8" s="9" t="s">
         <v>23</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>